<commit_message>
Added git link to the assessment
</commit_message>
<xml_diff>
--- a/Self Assessment Form - IUM.xlsx
+++ b/Self Assessment Form - IUM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\OneDrive\Desktop\Uni\3° anno\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\OneDrive\Desktop\Uni\3° anno\Progetto-IUM-TWEB.git\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0650448A-212F-49C7-A8C2-BFF9F8D95A15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55A58090-D765-410A-977D-8B246D651718}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13245" yWindow="600" windowWidth="23805" windowHeight="19260" xr2:uid="{9384817B-0988-A24F-9D66-74DAD74AC274}"/>
+    <workbookView xWindow="12990" yWindow="945" windowWidth="24405" windowHeight="19260" xr2:uid="{9384817B-0988-A24F-9D66-74DAD74AC274}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="65">
   <si>
     <t>Team Name</t>
   </si>
@@ -51,18 +51,9 @@
     <t>what</t>
   </si>
   <si>
-    <t>what we evaluate</t>
-  </si>
-  <si>
     <t>Comments and notes</t>
   </si>
   <si>
-    <t>Code style, naming, format (consistent format regarding class and variable naming as well as indentation, consistent format regarding class and variable naming as well as indentation)</t>
-  </si>
-  <si>
-    <t>Exception (Proper use and handling of  Exceptions in your code)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Code Organization (e.g. use of Javascript classes and modules, distribution of directories etc).  </t>
   </si>
   <si>
@@ -223,13 +214,28 @@
   </si>
   <si>
     <t>No</t>
+  </si>
+  <si>
+    <t>https://github.com/B-u-b-y/Jupiter-Notebooks</t>
+  </si>
+  <si>
+    <t>https://github.com/B-u-b-y/Footbal-Web-Page</t>
+  </si>
+  <si>
+    <t>https://github.com/B-u-b-y/Server-Flask</t>
+  </si>
+  <si>
+    <t>https://github.com/B-u-b-y/Server_Express</t>
+  </si>
+  <si>
+    <t>https://github.com/B-u-b-y/Spring-Boot-Server</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -375,6 +381,14 @@
       <color theme="1"/>
       <name val="Courier New"/>
       <family val="3"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -418,11 +432,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
@@ -524,23 +539,27 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Collegamento ipertestuale" xfId="2" builtinId="8"/>
     <cellStyle name="Default 1" xfId="1" xr:uid="{4CFB9B37-B9E9-0348-B0C6-CB853B61E7A3}"/>
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -865,20 +884,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="37" customFormat="1" ht="95.1" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="41" t="s">
-        <v>22</v>
-      </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
+      <c r="A1" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
     </row>
     <row r="2" spans="1:5" s="37" customFormat="1" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
+      <c r="A2" s="45" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
     </row>
     <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
@@ -932,14 +951,16 @@
     </row>
     <row r="11" spans="1:5" ht="33.75" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" s="24"/>
+        <v>21</v>
+      </c>
+      <c r="B11" s="46" t="s">
+        <v>60</v>
+      </c>
       <c r="C11" s="39" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="11" customFormat="1" ht="117" x14ac:dyDescent="0.35">
@@ -947,35 +968,37 @@
         <v>4</v>
       </c>
       <c r="B12" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="E12" s="10" t="s">
         <v>5</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="B13" s="28"/>
-    </row>
-    <row r="14" spans="1:5" ht="94.5" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="B13" s="28" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B14" s="29" t="s">
-        <v>7</v>
+        <v>63</v>
       </c>
       <c r="D14">
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B15" s="24" t="s">
-        <v>8</v>
+        <v>64</v>
       </c>
       <c r="D15">
         <v>3</v>
@@ -983,7 +1006,7 @@
     </row>
     <row r="16" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B16" s="24" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D16">
         <v>3</v>
@@ -991,12 +1014,12 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="18" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B21" s="36" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D21">
         <v>3</v>
@@ -1004,7 +1027,7 @@
     </row>
     <row r="22" spans="1:4" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B22" s="30" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D22">
         <v>3</v>
@@ -1012,25 +1035,25 @@
     </row>
     <row r="23" spans="1:4" ht="204.75" x14ac:dyDescent="0.25">
       <c r="B23" s="31" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D23" s="44" t="s">
-        <v>56</v>
+        <v>32</v>
+      </c>
+      <c r="D23" s="41" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B25" s="32"/>
       <c r="C25" s="4"/>
     </row>
     <row r="26" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B26" s="32" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C26" s="4"/>
       <c r="D26">
@@ -1039,7 +1062,7 @@
     </row>
     <row r="27" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B27" s="32" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C27" s="4"/>
       <c r="D27">
@@ -1048,7 +1071,7 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B28" s="31" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C28" s="4"/>
       <c r="D28">
@@ -1057,7 +1080,7 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B29" s="31" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C29" s="4"/>
       <c r="D29">
@@ -1069,14 +1092,14 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="18" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B33" s="23"/>
       <c r="C33" s="12"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B34" s="23" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C34" s="12"/>
       <c r="D34">
@@ -1085,7 +1108,7 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B35" s="23" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C35" s="12"/>
       <c r="D35">
@@ -1094,7 +1117,7 @@
     </row>
     <row r="36" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B36" s="40" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C36" s="21"/>
       <c r="D36">
@@ -1103,7 +1126,7 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B37" s="40" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C37" s="21"/>
       <c r="D37">
@@ -1112,7 +1135,7 @@
     </row>
     <row r="38" spans="1:4" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B38" s="1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C38" s="4"/>
       <c r="D38">
@@ -1121,25 +1144,25 @@
     </row>
     <row r="39" spans="1:4" ht="299.25" x14ac:dyDescent="0.25">
       <c r="B39" s="31" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D39" s="44" t="s">
-        <v>57</v>
+        <v>30</v>
+      </c>
+      <c r="D39" s="41" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="18" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B41" s="32"/>
       <c r="C41" s="4"/>
     </row>
     <row r="42" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B42" s="32" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C42" s="4"/>
       <c r="D42">
@@ -1148,7 +1171,7 @@
     </row>
     <row r="43" spans="1:4" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B43" s="32" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C43" s="4"/>
       <c r="D43">
@@ -1157,7 +1180,7 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B44" s="32" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C44" s="4"/>
       <c r="D44">
@@ -1166,7 +1189,7 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B45" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C45" s="4"/>
       <c r="D45">
@@ -1175,7 +1198,7 @@
     </row>
     <row r="46" spans="1:4" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B46" s="1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C46" s="4"/>
       <c r="D46">
@@ -1184,7 +1207,7 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B47" s="31" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C47" s="4"/>
       <c r="D47">
@@ -1193,7 +1216,7 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B48" s="31" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C48" s="4"/>
       <c r="D48">
@@ -1202,25 +1225,25 @@
     </row>
     <row r="49" spans="1:4" ht="126" x14ac:dyDescent="0.25">
       <c r="B49" s="31" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D49" s="44" t="s">
-        <v>59</v>
+        <v>36</v>
+      </c>
+      <c r="D49" s="41" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="18" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B50" s="23"/>
       <c r="C50" s="12"/>
     </row>
     <row r="51" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="B51" s="23" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C51" s="12"/>
       <c r="D51">
@@ -1229,7 +1252,7 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B52" s="23" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C52" s="12"/>
       <c r="D52">
@@ -1238,7 +1261,7 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B53" s="23" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C53" s="12"/>
       <c r="D53">
@@ -1247,7 +1270,7 @@
     </row>
     <row r="54" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B54" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C54" s="4"/>
       <c r="D54">
@@ -1256,7 +1279,7 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B55" s="33" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C55" s="21"/>
       <c r="D55">
@@ -1265,7 +1288,7 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B56" s="33" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C56" s="21"/>
       <c r="D56">
@@ -1274,23 +1297,23 @@
     </row>
     <row r="57" spans="1:4" ht="141.75" x14ac:dyDescent="0.25">
       <c r="B57" s="31" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C57" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="D57" s="44" t="s">
-        <v>60</v>
+        <v>49</v>
+      </c>
+      <c r="D57" s="41" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="18" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B62" s="30" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D62">
         <v>3</v>
@@ -1298,7 +1321,7 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B63" s="30" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D63">
         <v>3</v>
@@ -1306,35 +1329,35 @@
     </row>
     <row r="64" spans="1:4" ht="110.25" x14ac:dyDescent="0.25">
       <c r="B64" s="31" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C64" s="21" t="s">
-        <v>15</v>
-      </c>
-      <c r="D64" s="44" t="s">
-        <v>61</v>
+        <v>12</v>
+      </c>
+      <c r="D64" s="41" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="19" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="48" x14ac:dyDescent="0.3">
       <c r="A67" s="20"/>
       <c r="B67" s="30" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C67" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D67" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="68" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A68" s="34" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -1356,19 +1379,19 @@
     </row>
     <row r="71" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C71" s="4"/>
       <c r="D71" s="5"/>
     </row>
     <row r="72" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A72" s="35" t="s">
-        <v>17</v>
-      </c>
-      <c r="B72" s="45">
+        <v>14</v>
+      </c>
+      <c r="B72" s="42">
         <v>1</v>
       </c>
       <c r="C72" s="4"/>
@@ -1411,6 +1434,9 @@
       <formula1>"Yes, No"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="B11" r:id="rId1" xr:uid="{9CCD0920-F0A8-4082-8375-D21932A2296C}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
corrected rows content for error
</commit_message>
<xml_diff>
--- a/Self Assessment Form - IUM.xlsx
+++ b/Self Assessment Form - IUM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\OneDrive\Desktop\Uni\3° anno\Progetto-IUM-TWEB.git\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55A58090-D765-410A-977D-8B246D651718}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BD74B61-E62B-4781-AA6F-6392495BC73F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12990" yWindow="945" windowWidth="24405" windowHeight="19260" xr2:uid="{9384817B-0988-A24F-9D66-74DAD74AC274}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="64">
   <si>
     <t>Team Name</t>
   </si>
@@ -54,9 +54,6 @@
     <t>Comments and notes</t>
   </si>
   <si>
-    <t xml:space="preserve">Code Organization (e.g. use of Javascript classes and modules, distribution of directories etc).  </t>
-  </si>
-  <si>
     <t>instructions</t>
   </si>
   <si>
@@ -219,16 +216,16 @@
     <t>https://github.com/B-u-b-y/Jupiter-Notebooks</t>
   </si>
   <si>
-    <t>https://github.com/B-u-b-y/Footbal-Web-Page</t>
-  </si>
-  <si>
-    <t>https://github.com/B-u-b-y/Server-Flask</t>
-  </si>
-  <si>
-    <t>https://github.com/B-u-b-y/Server_Express</t>
-  </si>
-  <si>
-    <t>https://github.com/B-u-b-y/Spring-Boot-Server</t>
+    <t>Code style, naming, format (consistent format regarding class and variable naming as well as indentation, consistent format regarding class and variable naming as well as indentation)</t>
+  </si>
+  <si>
+    <t>Exception (Proper use and handling of Exceptions in your code)</t>
+  </si>
+  <si>
+    <t>Code Organization (e.g. use of Javascript classes and modules, distribution of directories etc).</t>
+  </si>
+  <si>
+    <t>what we evaluate</t>
   </si>
 </sst>
 </file>
@@ -545,6 +542,9 @@
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
     </xf>
@@ -552,9 +552,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -884,20 +881,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="37" customFormat="1" ht="95.1" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="43" t="s">
-        <v>19</v>
-      </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
+      <c r="A1" s="44" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
     </row>
     <row r="2" spans="1:5" s="37" customFormat="1" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="45" t="s">
-        <v>42</v>
-      </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
+      <c r="A2" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
     </row>
     <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
@@ -951,16 +948,16 @@
     </row>
     <row r="11" spans="1:5" ht="33.75" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="43" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="46" t="s">
-        <v>60</v>
-      </c>
-      <c r="C11" s="39" t="s">
-        <v>22</v>
-      </c>
       <c r="D11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="11" customFormat="1" ht="117" x14ac:dyDescent="0.35">
@@ -968,13 +965,13 @@
         <v>4</v>
       </c>
       <c r="B12" s="22" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>5</v>
@@ -982,23 +979,21 @@
     </row>
     <row r="13" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="B13" s="28" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="B13" s="28"/>
+    </row>
+    <row r="14" spans="1:5" ht="94.5" x14ac:dyDescent="0.25">
       <c r="B14" s="29" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D14">
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B15" s="24" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D15">
         <v>3</v>
@@ -1006,7 +1001,7 @@
     </row>
     <row r="16" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B16" s="24" t="s">
-        <v>6</v>
+        <v>62</v>
       </c>
       <c r="D16">
         <v>3</v>
@@ -1014,12 +1009,12 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="18" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B21" s="36" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D21">
         <v>3</v>
@@ -1027,7 +1022,7 @@
     </row>
     <row r="22" spans="1:4" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B22" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D22">
         <v>3</v>
@@ -1035,25 +1030,25 @@
     </row>
     <row r="23" spans="1:4" ht="204.75" x14ac:dyDescent="0.25">
       <c r="B23" s="31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D23" s="41" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B25" s="32"/>
       <c r="C25" s="4"/>
     </row>
     <row r="26" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B26" s="32" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C26" s="4"/>
       <c r="D26">
@@ -1062,7 +1057,7 @@
     </row>
     <row r="27" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B27" s="32" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C27" s="4"/>
       <c r="D27">
@@ -1071,7 +1066,7 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B28" s="31" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C28" s="4"/>
       <c r="D28">
@@ -1080,7 +1075,7 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B29" s="31" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C29" s="4"/>
       <c r="D29">
@@ -1092,14 +1087,14 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="18" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B33" s="23"/>
       <c r="C33" s="12"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B34" s="23" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C34" s="12"/>
       <c r="D34">
@@ -1108,7 +1103,7 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B35" s="23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C35" s="12"/>
       <c r="D35">
@@ -1117,7 +1112,7 @@
     </row>
     <row r="36" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B36" s="40" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C36" s="21"/>
       <c r="D36">
@@ -1126,7 +1121,7 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B37" s="40" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C37" s="21"/>
       <c r="D37">
@@ -1135,7 +1130,7 @@
     </row>
     <row r="38" spans="1:4" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B38" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C38" s="4"/>
       <c r="D38">
@@ -1144,25 +1139,25 @@
     </row>
     <row r="39" spans="1:4" ht="299.25" x14ac:dyDescent="0.25">
       <c r="B39" s="31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D39" s="41" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="18" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B41" s="32"/>
       <c r="C41" s="4"/>
     </row>
     <row r="42" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B42" s="32" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C42" s="4"/>
       <c r="D42">
@@ -1171,7 +1166,7 @@
     </row>
     <row r="43" spans="1:4" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B43" s="32" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C43" s="4"/>
       <c r="D43">
@@ -1180,7 +1175,7 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B44" s="32" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C44" s="4"/>
       <c r="D44">
@@ -1189,7 +1184,7 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B45" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C45" s="4"/>
       <c r="D45">
@@ -1198,7 +1193,7 @@
     </row>
     <row r="46" spans="1:4" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B46" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C46" s="4"/>
       <c r="D46">
@@ -1207,7 +1202,7 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B47" s="31" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C47" s="4"/>
       <c r="D47">
@@ -1216,7 +1211,7 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B48" s="31" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C48" s="4"/>
       <c r="D48">
@@ -1225,25 +1220,25 @@
     </row>
     <row r="49" spans="1:4" ht="126" x14ac:dyDescent="0.25">
       <c r="B49" s="31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D49" s="41" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B50" s="23"/>
       <c r="C50" s="12"/>
     </row>
     <row r="51" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="B51" s="23" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C51" s="12"/>
       <c r="D51">
@@ -1252,7 +1247,7 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B52" s="23" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C52" s="12"/>
       <c r="D52">
@@ -1261,7 +1256,7 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B53" s="23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C53" s="12"/>
       <c r="D53">
@@ -1270,7 +1265,7 @@
     </row>
     <row r="54" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B54" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C54" s="4"/>
       <c r="D54">
@@ -1279,7 +1274,7 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B55" s="33" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C55" s="21"/>
       <c r="D55">
@@ -1288,7 +1283,7 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B56" s="33" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C56" s="21"/>
       <c r="D56">
@@ -1297,23 +1292,23 @@
     </row>
     <row r="57" spans="1:4" ht="141.75" x14ac:dyDescent="0.25">
       <c r="B57" s="31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C57" s="21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D57" s="41" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="18" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B62" s="30" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D62">
         <v>3</v>
@@ -1321,7 +1316,7 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B63" s="30" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D63">
         <v>3</v>
@@ -1329,35 +1324,35 @@
     </row>
     <row r="64" spans="1:4" ht="110.25" x14ac:dyDescent="0.25">
       <c r="B64" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="C64" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="C64" s="21" t="s">
-        <v>12</v>
-      </c>
       <c r="D64" s="41" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="48" x14ac:dyDescent="0.3">
       <c r="A67" s="20"/>
       <c r="B67" s="30" t="s">
+        <v>16</v>
+      </c>
+      <c r="C67" t="s">
         <v>17</v>
       </c>
-      <c r="C67" t="s">
-        <v>18</v>
-      </c>
       <c r="D67" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="68" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A68" s="34" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -1379,17 +1374,17 @@
     </row>
     <row r="71" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C71" s="4"/>
       <c r="D71" s="5"/>
     </row>
     <row r="72" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A72" s="35" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B72" s="42">
         <v>1</v>

</xml_diff>